<commit_message>
feat(config): add skill definitions and generated tables
</commit_message>
<xml_diff>
--- a/GameConfig/Datas/__tables__.xlsx
+++ b/GameConfig/Datas/__tables__.xlsx
@@ -1331,6 +1331,43 @@
       <x:c r="K16"/>
       <x:c r="L16"/>
     </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="1"/>
+      <x:c r="B17" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">skill.TbSkill</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Skill</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="1" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E17" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">skill.xlsx</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F17" s="1"/>
+      <x:c r="G17" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">map</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H17" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">c</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I17" s="1" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">技能配置</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>